<commit_message>
LRP: self-serve advertising and AI article review
Owner: advertising is self-serve on the site, and article review becomes
an AI agent once trusted. The plan drops commissioned account executives
and per-town reviewers for small partnerships and editorial standards
teams (1 per 1,000 towns each) and adds an AI review pass to the cost
per story. Base case: EBITDA positive in FY2028, about $7.7M needed.
Code is unchanged: Tier 3 still needs a person (Rule 5).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VYAkBQdsKV9f29chT2ka2T
</commit_message>
<xml_diff>
--- a/docs/finance/TownCore-LRP.xlsx
+++ b/docs/finance/TownCore-LRP.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="358">
   <si>
     <t xml:space="preserve">TownCore long-range plan, FY2027-FY2031</t>
   </si>
@@ -187,7 +187,7 @@
     <t xml:space="preserve">Share that pass readiness (Rule 7)</t>
   </si>
   <si>
-    <t xml:space="preserve">Owner plan: every town. Rule 7 still stops a town below 3 real items a day (10 for large), and today almost none pass: Boca makes about 0.8 a day, Delray 0.53. Reaching 100% needs many more sources per town or a lower bar. Set lower to see the plan without that work.</t>
+    <t xml:space="preserve">Owner, 2026-10-17: every town in America can make 3 real items a day; Rule 7 is the target we build sources toward. Today Boca makes about 0.8 a day and Delray 0.53, so the source work continues. Set lower to see the plan if some towns stay short.</t>
   </si>
   <si>
     <t xml:space="preserve">Share allowed by the naming rule</t>
@@ -430,7 +430,7 @@
     <t xml:space="preserve">$/story</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimate for writer + separate fact-check calls; verify against current Anthropic pricing (CLAUDE.md §8). Scaled by unit cost multiplier.</t>
+    <t xml:space="preserve">Writer, separate fact-check and an AI review pass (owner: article review becomes an AI agent). Measured ~$0.10 for writer + fact-check on repo pricing; verify against current Anthropic pricing (CLAUDE.md §8). Scaled by unit cost multiplier.</t>
   </si>
   <si>
     <t xml:space="preserve">AI overhead per town per day</t>
@@ -529,19 +529,19 @@
     <t xml:space="preserve">Sales commission on direct-sold revenue</t>
   </si>
   <si>
-    <t xml:space="preserve">Paid on banners, newsletter and category sponsorships. Estimate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Towns per editorial reviewer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reviewers approve Tier 3 items and samples (§7). Estimate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Towns per local account executive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clustered towns share sales effort (§10a). Estimate.</t>
+    <t xml:space="preserve">Owner: advertisers sign up and pay on the site; no commissioned sales force.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Towns per editorial standards editor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner, 2026-10-17: article review becomes an AI agent once we trust it. A small team audits the agent, handles corrections and reader reports. Until the agent ships, Tier 3 still needs a person (Rule 5).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Towns per advertiser partnerships manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner, 2026-10-17: sales are self-serve on the site. A small team handles regional and multi-town advertisers.</t>
   </si>
   <si>
     <t xml:space="preserve">Towns per support and success rep</t>
@@ -556,10 +556,10 @@
     <t xml:space="preserve">Engineering</t>
   </si>
   <si>
-    <t xml:space="preserve">Editorial reviewer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Account executive (base)</t>
+    <t xml:space="preserve">Editorial standards and launch operations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advertiser partnerships</t>
   </si>
   <si>
     <t xml:space="preserve">Support and success</t>
@@ -646,7 +646,7 @@
     <t xml:space="preserve">Equity raised</t>
   </si>
   <si>
-    <t xml:space="preserve">Plan: $25M in FY2027 and $35M in FY2028, sized to the every-town launch pace with a buffer. Adjust to keep cash above zero.</t>
+    <t xml:space="preserve">Plan: $10M in FY2027, the ~$7.7M the every-town plan needs plus a buffer. Adjust to keep cash above zero.</t>
   </si>
   <si>
     <t xml:space="preserve">Town rollout</t>
@@ -799,10 +799,10 @@
     <t xml:space="preserve">Town-level people and acquisition costs ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">Editorial review (share of a reviewer)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Local sales (share of an AE) + commission</t>
+    <t xml:space="preserve">Editorial standards (share)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advertiser partnerships (share) + commission</t>
   </si>
   <si>
     <t xml:space="preserve">Support and success (share)</t>
@@ -868,10 +868,7 @@
     <t xml:space="preserve">Heads (year end)</t>
   </si>
   <si>
-    <t xml:space="preserve">Editorial reviewers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Account executives</t>
+    <t xml:space="preserve">Editorial standards</t>
   </si>
   <si>
     <t xml:space="preserve">Launch operations</t>
@@ -910,10 +907,10 @@
     <t xml:space="preserve">Operating expenses</t>
   </si>
   <si>
-    <t xml:space="preserve">Editorial review (people)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sales (people)</t>
+    <t xml:space="preserve">Editorial standards (people)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advertiser partnerships (people)</t>
   </si>
   <si>
     <t xml:space="preserve">Sales commission</t>
@@ -1883,23 +1880,23 @@
       <c r="B10" s="2"/>
       <c r="C10" s="10" t="n">
         <f aca="false">'P&amp;L'!C8</f>
-        <v>0.431548852760639</v>
+        <v>0.400052059525826</v>
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">'P&amp;L'!D8</f>
-        <v>0.799502416256723</v>
+        <v>0.789260818887664</v>
       </c>
       <c r="E10" s="10" t="n">
         <f aca="false">'P&amp;L'!E8</f>
-        <v>0.88225003205724</v>
+        <v>0.876673851609431</v>
       </c>
       <c r="F10" s="10" t="n">
         <f aca="false">'P&amp;L'!F8</f>
-        <v>0.918154757640337</v>
+        <v>0.914613415716302</v>
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">'P&amp;L'!G8</f>
-        <v>0.936222688325491</v>
+        <v>0.933708003592243</v>
       </c>
       <c r="H10" s="2"/>
     </row>
@@ -1910,23 +1907,23 @@
       <c r="B11" s="2"/>
       <c r="C11" s="9" t="n">
         <f aca="false">'P&amp;L'!C16</f>
-        <v>-18714272.68496</v>
+        <v>-7576935.88496</v>
       </c>
       <c r="D11" s="9" t="n">
         <f aca="false">'P&amp;L'!D16</f>
-        <v>-21529601.343104</v>
+        <v>1710094.032896</v>
       </c>
       <c r="E11" s="9" t="n">
         <f aca="false">'P&amp;L'!E16</f>
-        <v>-9655829.95082656</v>
+        <v>28895708.3674734</v>
       </c>
       <c r="F11" s="9" t="n">
         <f aca="false">'P&amp;L'!F16</f>
-        <v>22598678.7557132</v>
+        <v>69401273.7358492</v>
       </c>
       <c r="G11" s="9" t="n">
         <f aca="false">'P&amp;L'!G16</f>
-        <v>54040935.9844372</v>
+        <v>103097468.531385</v>
       </c>
       <c r="H11" s="2"/>
     </row>
@@ -1937,23 +1934,23 @@
       <c r="B12" s="2"/>
       <c r="C12" s="10" t="n">
         <f aca="false">'P&amp;L'!C17</f>
-        <v>-9.85899237790985</v>
+        <v>-3.99165676354426</v>
       </c>
       <c r="D12" s="10" t="n">
         <f aca="false">'P&amp;L'!D17</f>
-        <v>-1.25443913462188</v>
+        <v>0.0996399721741811</v>
       </c>
       <c r="E12" s="10" t="n">
         <f aca="false">'P&amp;L'!E17</f>
-        <v>-0.193630303722282</v>
+        <v>0.579451462583535</v>
       </c>
       <c r="F12" s="10" t="n">
         <f aca="false">'P&amp;L'!F17</f>
-        <v>0.250045659732808</v>
+        <v>0.76789831233786</v>
       </c>
       <c r="G12" s="10" t="n">
         <f aca="false">'P&amp;L'!G17</f>
-        <v>0.430419265417366</v>
+        <v>0.82113930603363</v>
       </c>
       <c r="H12" s="2"/>
     </row>
@@ -1964,23 +1961,23 @@
       <c r="B13" s="2"/>
       <c r="C13" s="9" t="n">
         <f aca="false">'P&amp;L'!C25</f>
-        <v>-18892606.0182933</v>
+        <v>-7614435.88496</v>
       </c>
       <c r="D13" s="9" t="n">
         <f aca="false">'P&amp;L'!D25</f>
-        <v>-21872101.343104</v>
+        <v>1645094.032896</v>
       </c>
       <c r="E13" s="9" t="n">
         <f aca="false">'P&amp;L'!E25</f>
-        <v>-10129163.2841599</v>
+        <v>23097241.7386211</v>
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">'P&amp;L'!F25</f>
-        <v>22303678.7557132</v>
+        <v>52012205.3018869</v>
       </c>
       <c r="G13" s="9" t="n">
         <f aca="false">'P&amp;L'!G25</f>
-        <v>47580124.9607889</v>
+        <v>77303101.3985385</v>
       </c>
       <c r="H13" s="2"/>
     </row>
@@ -1991,23 +1988,23 @@
       <c r="B14" s="2"/>
       <c r="C14" s="9" t="n">
         <f aca="false">'Cash Flow'!C13</f>
-        <v>5943781.51784</v>
+        <v>2503618.31784</v>
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">'Cash Flow'!D13</f>
-        <v>18463744.043856</v>
+        <v>3673276.219856</v>
       </c>
       <c r="E14" s="9" t="n">
         <f aca="false">'Cash Flow'!E13</f>
-        <v>7434275.54830025</v>
+        <v>25806046.0804145</v>
       </c>
       <c r="F14" s="9" t="n">
         <f aca="false">'Cash Flow'!F13</f>
-        <v>28817628.523519</v>
+        <v>76654592.2684737</v>
       </c>
       <c r="G14" s="9" t="n">
         <f aca="false">'Cash Flow'!G13</f>
-        <v>75473307.8062485</v>
+        <v>152921581.322286</v>
       </c>
       <c r="H14" s="2"/>
     </row>
@@ -2018,23 +2015,23 @@
       <c r="B15" s="2"/>
       <c r="C15" s="9" t="n">
         <f aca="false">KPIs!C22</f>
-        <v>33780959.8039639</v>
+        <v>50953224.2039639</v>
       </c>
       <c r="D15" s="9" t="n">
         <f aca="false">KPIs!D22</f>
-        <v>66863868.3138088</v>
+        <v>100693439.181809</v>
       </c>
       <c r="E15" s="9" t="n">
         <f aca="false">KPIs!E22</f>
-        <v>92357578.2246254</v>
+        <v>139253415.301025</v>
       </c>
       <c r="F15" s="9" t="n">
         <f aca="false">KPIs!F22</f>
-        <v>89083676.518476</v>
+        <v>135044089.780024</v>
       </c>
       <c r="G15" s="9" t="n">
         <f aca="false">KPIs!G22</f>
-        <v>86343208.4565014</v>
+        <v>131691005.841481</v>
       </c>
       <c r="H15" s="2"/>
     </row>
@@ -2229,7 +2226,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2241,7 +2238,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2285,7 +2282,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -2297,7 +2294,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="33" t="n">
@@ -2378,7 +2375,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="33" t="n">
@@ -2405,7 +2402,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B10" s="16"/>
       <c r="C10" s="16"/>
@@ -2417,7 +2414,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="33" t="n">
@@ -2444,7 +2441,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="42" t="n">
@@ -2471,7 +2468,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -2510,7 +2507,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="37" t="n">
@@ -2542,23 +2539,23 @@
       <c r="B16" s="2"/>
       <c r="C16" s="34" t="n">
         <f aca="false">'P&amp;L'!C8</f>
-        <v>0.431548852760639</v>
+        <v>0.400052059525826</v>
       </c>
       <c r="D16" s="34" t="n">
         <f aca="false">'P&amp;L'!D8</f>
-        <v>0.799502416256723</v>
+        <v>0.789260818887664</v>
       </c>
       <c r="E16" s="34" t="n">
         <f aca="false">'P&amp;L'!E8</f>
-        <v>0.88225003205724</v>
+        <v>0.876673851609431</v>
       </c>
       <c r="F16" s="34" t="n">
         <f aca="false">'P&amp;L'!F8</f>
-        <v>0.918154757640337</v>
+        <v>0.914613415716302</v>
       </c>
       <c r="G16" s="34" t="n">
         <f aca="false">'P&amp;L'!G8</f>
-        <v>0.936222688325491</v>
+        <v>0.933708003592243</v>
       </c>
       <c r="H16" s="2"/>
     </row>
@@ -2569,23 +2566,23 @@
       <c r="B17" s="2"/>
       <c r="C17" s="37" t="n">
         <f aca="false">'P&amp;L'!C16</f>
-        <v>-18714272.68496</v>
+        <v>-7576935.88496</v>
       </c>
       <c r="D17" s="37" t="n">
         <f aca="false">'P&amp;L'!D16</f>
-        <v>-21529601.343104</v>
+        <v>1710094.032896</v>
       </c>
       <c r="E17" s="37" t="n">
         <f aca="false">'P&amp;L'!E16</f>
-        <v>-9655829.95082656</v>
+        <v>28895708.3674734</v>
       </c>
       <c r="F17" s="37" t="n">
         <f aca="false">'P&amp;L'!F16</f>
-        <v>22598678.7557132</v>
+        <v>69401273.7358492</v>
       </c>
       <c r="G17" s="37" t="n">
         <f aca="false">'P&amp;L'!G16</f>
-        <v>54040935.9844372</v>
+        <v>103097468.531385</v>
       </c>
       <c r="H17" s="2"/>
     </row>
@@ -2596,23 +2593,23 @@
       <c r="B18" s="2"/>
       <c r="C18" s="34" t="n">
         <f aca="false">'P&amp;L'!C17</f>
-        <v>-9.85899237790985</v>
+        <v>-3.99165676354426</v>
       </c>
       <c r="D18" s="34" t="n">
         <f aca="false">'P&amp;L'!D17</f>
-        <v>-1.25443913462188</v>
+        <v>0.0996399721741811</v>
       </c>
       <c r="E18" s="34" t="n">
         <f aca="false">'P&amp;L'!E17</f>
-        <v>-0.193630303722282</v>
+        <v>0.579451462583535</v>
       </c>
       <c r="F18" s="34" t="n">
         <f aca="false">'P&amp;L'!F17</f>
-        <v>0.250045659732808</v>
+        <v>0.76789831233786</v>
       </c>
       <c r="G18" s="34" t="n">
         <f aca="false">'P&amp;L'!G17</f>
-        <v>0.430419265417366</v>
+        <v>0.82113930603363</v>
       </c>
       <c r="H18" s="2"/>
     </row>
@@ -2623,135 +2620,135 @@
       <c r="B19" s="2"/>
       <c r="C19" s="37" t="n">
         <f aca="false">'Cash Flow'!C13</f>
-        <v>5943781.51784</v>
+        <v>2503618.31784</v>
       </c>
       <c r="D19" s="37" t="n">
         <f aca="false">'Cash Flow'!D13</f>
-        <v>18463744.043856</v>
+        <v>3673276.219856</v>
       </c>
       <c r="E19" s="37" t="n">
         <f aca="false">'Cash Flow'!E13</f>
-        <v>7434275.54830025</v>
+        <v>25806046.0804145</v>
       </c>
       <c r="F19" s="37" t="n">
         <f aca="false">'Cash Flow'!F13</f>
-        <v>28817628.523519</v>
+        <v>76654592.2684737</v>
       </c>
       <c r="G19" s="37" t="n">
         <f aca="false">'Cash Flow'!G13</f>
-        <v>75473307.8062485</v>
+        <v>152921581.322286</v>
       </c>
       <c r="H19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="34" t="n">
         <f aca="false">IF('P&amp;L'!C5=0,0,Costs!C6/'P&amp;L'!C5)</f>
-        <v>0.270203259179239</v>
+        <v>0.301700052414052</v>
       </c>
       <c r="D20" s="34" t="n">
         <f aca="false">IF('P&amp;L'!D5=0,0,Costs!D6/'P&amp;L'!D5)</f>
-        <v>0.0878601503235732</v>
+        <v>0.0981017476926319</v>
       </c>
       <c r="E20" s="34" t="n">
         <f aca="false">IF('P&amp;L'!E5=0,0,Costs!E6/'P&amp;L'!E5)</f>
-        <v>0.0478366835485996</v>
+        <v>0.0534128639964081</v>
       </c>
       <c r="F20" s="34" t="n">
         <f aca="false">IF('P&amp;L'!F5=0,0,Costs!F6/'P&amp;L'!F5)</f>
-        <v>0.0303803032457523</v>
+        <v>0.0339216451697874</v>
       </c>
       <c r="G20" s="34" t="n">
         <f aca="false">IF('P&amp;L'!G5=0,0,Costs!G6/'P&amp;L'!G5)</f>
-        <v>0.0215728631694795</v>
+        <v>0.024087547902728</v>
       </c>
       <c r="H20" s="17" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="37" t="n">
         <f aca="false">Costs!C22+Costs!C23+Costs!C24+Costs!C21+Assumptions!C$97+Costs!C26</f>
-        <v>1633250</v>
+        <v>1126250</v>
       </c>
       <c r="D21" s="37" t="n">
         <f aca="false">Costs!D22+Costs!D23+Costs!D24+Costs!D21+Assumptions!D$97+Costs!D26</f>
-        <v>2902125</v>
+        <v>1903125</v>
       </c>
       <c r="E21" s="37" t="n">
         <f aca="false">Costs!E22+Costs!E23+Costs!E24+Costs!E21+Assumptions!E$97+Costs!E26</f>
-        <v>4358628.75</v>
+        <v>2975628.75</v>
       </c>
       <c r="F21" s="37" t="n">
         <f aca="false">Costs!F22+Costs!F23+Costs!F24+Costs!F21+Assumptions!F$97+Costs!F26</f>
-        <v>5708476.4375</v>
+        <v>4355476.4375</v>
       </c>
       <c r="G21" s="37" t="n">
         <f aca="false">Costs!G22+Costs!G23+Costs!G24+Costs!G21+Assumptions!G$97+Costs!G26</f>
-        <v>7166241.820375</v>
+        <v>5822241.820375</v>
       </c>
       <c r="H21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="37" t="n">
         <f aca="false">Rollout!C7/'Unit Economics'!$G$7*'Unit Economics'!$G$42-C21</f>
-        <v>33780959.8039639</v>
+        <v>50953224.2039639</v>
       </c>
       <c r="D22" s="37" t="n">
         <f aca="false">Rollout!D7/'Unit Economics'!$G$7*'Unit Economics'!$G$42-D21</f>
-        <v>66863868.3138088</v>
+        <v>100693439.181809</v>
       </c>
       <c r="E22" s="37" t="n">
         <f aca="false">Rollout!E7/'Unit Economics'!$G$7*'Unit Economics'!$G$42-E21</f>
-        <v>92357578.2246254</v>
+        <v>139253415.301025</v>
       </c>
       <c r="F22" s="37" t="n">
         <f aca="false">Rollout!F7/'Unit Economics'!$G$7*'Unit Economics'!$G$42-F21</f>
-        <v>89083676.518476</v>
+        <v>135044089.780024</v>
       </c>
       <c r="G22" s="37" t="n">
         <f aca="false">Rollout!G7/'Unit Economics'!$G$7*'Unit Economics'!$G$42-G21</f>
-        <v>86343208.4565014</v>
+        <v>131691005.841481</v>
       </c>
       <c r="H22" s="17" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="33" t="n">
         <f aca="false">IF('Unit Economics'!$G$42&lt;=0,0,C21/('Unit Economics'!$G$42/'Unit Economics'!$G$7))</f>
-        <v>138.355480105943</v>
+        <v>64.8768070654376</v>
       </c>
       <c r="D23" s="33" t="n">
         <f aca="false">IF('Unit Economics'!$G$42&lt;=0,0,D21/('Unit Economics'!$G$42/'Unit Economics'!$G$7))</f>
-        <v>245.844113088908</v>
+        <v>109.628122926891</v>
       </c>
       <c r="E23" s="33" t="n">
         <f aca="false">IF('Unit Economics'!$G$42&lt;=0,0,E21/('Unit Economics'!$G$42/'Unit Economics'!$G$7))</f>
-        <v>369.227107491085</v>
+        <v>171.408916592337</v>
       </c>
       <c r="F23" s="33" t="n">
         <f aca="false">IF('Unit Economics'!$G$42&lt;=0,0,F21/('Unit Economics'!$G$42/'Unit Economics'!$G$7))</f>
-        <v>483.575079249211</v>
+        <v>250.894032864592</v>
       </c>
       <c r="G23" s="33" t="n">
         <f aca="false">IF('Unit Economics'!$G$42&lt;=0,0,G21/('Unit Economics'!$G$42/'Unit Economics'!$G$7))</f>
-        <v>607.064948791224</v>
+        <v>335.385979372956</v>
       </c>
       <c r="H23" s="2"/>
     </row>
@@ -2767,7 +2764,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B25" s="16"/>
       <c r="C25" s="16"/>
@@ -2779,7 +2776,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="9" t="n">
@@ -2794,12 +2791,12 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="9" t="n">
         <f aca="false">'Unit Economics'!G42</f>
-        <v>10978.4050392288</v>
+        <v>16144.6370032288</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
@@ -2809,12 +2806,12 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="10" t="n">
         <f aca="false">'Unit Economics'!G43</f>
-        <v>0.612127686524311</v>
+        <v>0.900183520579547</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -2824,7 +2821,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="9" t="n">
@@ -2839,29 +2836,29 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="41" t="n">
         <f aca="false">IFERROR(MATCH(TRUE(),INDEX('Unit Economics'!C45:G45&gt;0,0),0),"After Age 5")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="17" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2" t="str">
         <f aca="false">IFERROR(INDEX(C4:G4,MATCH(TRUE(),INDEX(C17:G17&gt;0,0),0)),"Not by FY2031")</f>
-        <v>2030</v>
+        <v>2028</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -2871,12 +2868,12 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="9" t="n">
         <f aca="false">'Cash Flow'!C17</f>
-        <v>52815724.4516998</v>
+        <v>7746381.68216</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
@@ -3939,7 +3936,7 @@
         <v>132</v>
       </c>
       <c r="C58" s="31" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
@@ -4221,7 +4218,7 @@
       </c>
       <c r="B75" s="17"/>
       <c r="C75" s="23" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D75" s="2"/>
       <c r="E75" s="2"/>
@@ -4239,7 +4236,7 @@
         <v>49</v>
       </c>
       <c r="C76" s="24" t="n">
-        <v>40</v>
+        <v>1000</v>
       </c>
       <c r="D76" s="2"/>
       <c r="E76" s="2"/>
@@ -4257,7 +4254,7 @@
         <v>49</v>
       </c>
       <c r="C77" s="24" t="n">
-        <v>30</v>
+        <v>1000</v>
       </c>
       <c r="D77" s="2"/>
       <c r="E77" s="2"/>
@@ -4817,10 +4814,10 @@
         <v>185</v>
       </c>
       <c r="C109" s="32" t="n">
-        <v>25000000</v>
+        <v>10000000</v>
       </c>
       <c r="D109" s="32" t="n">
-        <v>35000000</v>
+        <v>0</v>
       </c>
       <c r="E109" s="32" t="n">
         <v>0</v>
@@ -5753,23 +5750,23 @@
       <c r="B29" s="2"/>
       <c r="C29" s="37" t="n">
         <f aca="false">MIN(Assumptions!$C$60,Assumptions!$F$26*Assumptions!$C$58+Assumptions!$C$59)*Assumptions!$F$10*365*C8</f>
-        <v>170.966</v>
+        <v>190.895</v>
       </c>
       <c r="D29" s="37" t="n">
         <f aca="false">MIN(Assumptions!$C$60,Assumptions!$F$26*Assumptions!$C$58+Assumptions!$C$59)*Assumptions!$F$10*365*D8</f>
-        <v>331.67404</v>
+        <v>370.3363</v>
       </c>
       <c r="E29" s="37" t="n">
         <f aca="false">MIN(Assumptions!$C$60,Assumptions!$F$26*Assumptions!$C$58+Assumptions!$C$59)*Assumptions!$F$10*365*E8</f>
-        <v>324.8354</v>
+        <v>362.7005</v>
       </c>
       <c r="F29" s="37" t="n">
         <f aca="false">MIN(Assumptions!$C$60,Assumptions!$F$26*Assumptions!$C$58+Assumptions!$C$59)*Assumptions!$F$10*365*F8</f>
-        <v>321.41608</v>
+        <v>358.8826</v>
       </c>
       <c r="G29" s="37" t="n">
         <f aca="false">MIN(Assumptions!$C$60,Assumptions!$F$26*Assumptions!$C$58+Assumptions!$C$59)*Assumptions!$F$10*365*G8</f>
-        <v>317.99676</v>
+        <v>355.0647</v>
       </c>
       <c r="H29" s="17" t="s">
         <v>247</v>
@@ -5892,23 +5889,23 @@
       <c r="B34" s="2"/>
       <c r="C34" s="38" t="n">
         <f aca="false">SUM(C29:C33)</f>
-        <v>344.67670832</v>
+        <v>364.60570832</v>
       </c>
       <c r="D34" s="38" t="n">
         <f aca="false">SUM(D29:D33)</f>
-        <v>787.351986048</v>
+        <v>826.014246048</v>
       </c>
       <c r="E34" s="38" t="n">
         <f aca="false">SUM(E29:E33)</f>
-        <v>878.24312256</v>
+        <v>916.10822256</v>
       </c>
       <c r="F34" s="38" t="n">
         <f aca="false">SUM(F29:F33)</f>
-        <v>948.889874784</v>
+        <v>986.356394784</v>
       </c>
       <c r="G34" s="38" t="n">
         <f aca="false">SUM(G29:G33)</f>
-        <v>1008.0242135712</v>
+        <v>1045.0921535712</v>
       </c>
       <c r="H34" s="2"/>
     </row>
@@ -5919,23 +5916,23 @@
       <c r="B35" s="2"/>
       <c r="C35" s="28" t="n">
         <f aca="false">C25-C34</f>
-        <v>288.05437168</v>
+        <v>268.12537168</v>
       </c>
       <c r="D35" s="28" t="n">
         <f aca="false">D25-D34</f>
-        <v>4300.827245952</v>
+        <v>4262.164985952</v>
       </c>
       <c r="E35" s="28" t="n">
         <f aca="false">E25-E34</f>
-        <v>10142.88243744</v>
+        <v>10105.01733744</v>
       </c>
       <c r="F35" s="28" t="n">
         <f aca="false">F25-F34</f>
-        <v>14029.540689216</v>
+        <v>13992.074169216</v>
       </c>
       <c r="G35" s="28" t="n">
         <f aca="false">G25-G34</f>
-        <v>16926.8042232288</v>
+        <v>16889.7362832288</v>
       </c>
       <c r="H35" s="2"/>
     </row>
@@ -5946,23 +5943,23 @@
       <c r="B36" s="2"/>
       <c r="C36" s="34" t="n">
         <f aca="false">IF(C25=0,0,C35/C25)</f>
-        <v>0.455255606663103</v>
+        <v>0.423758813428289</v>
       </c>
       <c r="D36" s="34" t="n">
         <f aca="false">IF(D25=0,0,D35/D25)</f>
-        <v>0.845258598381072</v>
+        <v>0.837660151424477</v>
       </c>
       <c r="E36" s="34" t="n">
         <f aca="false">IF(E25=0,0,E35/E25)</f>
-        <v>0.920312755917827</v>
+        <v>0.916877072348679</v>
       </c>
       <c r="F36" s="34" t="n">
         <f aca="false">IF(F25=0,0,F35/F25)</f>
-        <v>0.936649579491685</v>
+        <v>0.934148214623055</v>
       </c>
       <c r="G36" s="34" t="n">
         <f aca="false">IF(G25=0,0,G35/G25)</f>
-        <v>0.943795157164545</v>
+        <v>0.941728343973071</v>
       </c>
       <c r="H36" s="2"/>
     </row>
@@ -5985,23 +5982,23 @@
       <c r="B38" s="2"/>
       <c r="C38" s="37" t="n">
         <f aca="false">Assumptions!$C$83*(1+Assumptions!$C$73)/Assumptions!$C$76*C8</f>
-        <v>1093.75</v>
+        <v>43.75</v>
       </c>
       <c r="D38" s="37" t="n">
         <f aca="false">Assumptions!$C$83*(1+Assumptions!$C$73)/Assumptions!$C$76*D8</f>
-        <v>2121.875</v>
+        <v>84.875</v>
       </c>
       <c r="E38" s="37" t="n">
         <f aca="false">Assumptions!$C$83*(1+Assumptions!$C$73)/Assumptions!$C$76*E8</f>
-        <v>2078.125</v>
+        <v>83.125</v>
       </c>
       <c r="F38" s="37" t="n">
         <f aca="false">Assumptions!$C$83*(1+Assumptions!$C$73)/Assumptions!$C$76*F8</f>
-        <v>2056.25</v>
+        <v>82.25</v>
       </c>
       <c r="G38" s="37" t="n">
         <f aca="false">Assumptions!$C$83*(1+Assumptions!$C$73)/Assumptions!$C$76*G8</f>
-        <v>2034.375</v>
+        <v>81.375</v>
       </c>
       <c r="H38" s="2"/>
     </row>
@@ -6012,23 +6009,23 @@
       <c r="B39" s="2"/>
       <c r="C39" s="37" t="n">
         <f aca="false">Assumptions!$C$84*(1+Assumptions!$C$73)/Assumptions!$C$77*C8+C27*Assumptions!$C$75</f>
-        <v>1372.22876666667</v>
+        <v>40.625</v>
       </c>
       <c r="D39" s="37" t="n">
         <f aca="false">Assumptions!$C$84*(1+Assumptions!$C$73)/Assumptions!$C$77*D8+D27*Assumptions!$C$75</f>
-        <v>2849.71928533333</v>
+        <v>78.8125</v>
       </c>
       <c r="E39" s="37" t="n">
         <f aca="false">Assumptions!$C$84*(1+Assumptions!$C$73)/Assumptions!$C$77*E8+E27*Assumptions!$C$75</f>
-        <v>3037.42448666667</v>
+        <v>77.1875</v>
       </c>
       <c r="F39" s="37" t="n">
         <f aca="false">Assumptions!$C$84*(1+Assumptions!$C$73)/Assumptions!$C$77*F8+F27*Assumptions!$C$75</f>
-        <v>3220.49718333333</v>
+        <v>76.375</v>
       </c>
       <c r="G39" s="37" t="n">
         <f aca="false">Assumptions!$C$84*(1+Assumptions!$C$73)/Assumptions!$C$77*G8+G27*Assumptions!$C$75</f>
-        <v>3325.862404</v>
+        <v>75.5625</v>
       </c>
       <c r="H39" s="2"/>
     </row>
@@ -6093,23 +6090,23 @@
       <c r="B42" s="2"/>
       <c r="C42" s="38" t="n">
         <f aca="false">C35-SUM(C38:C41)</f>
-        <v>-2561.48672832</v>
+        <v>-199.811961653333</v>
       </c>
       <c r="D42" s="38" t="n">
         <f aca="false">D35-SUM(D38:D41)</f>
-        <v>-1380.567886048</v>
+        <v>3388.67663928533</v>
       </c>
       <c r="E42" s="38" t="n">
         <f aca="false">E35-SUM(E38:E41)</f>
-        <v>4365.24259744</v>
+        <v>9282.61448410667</v>
       </c>
       <c r="F42" s="38" t="n">
         <f aca="false">F35-SUM(F38:F41)</f>
-        <v>8126.858239216</v>
+        <v>13207.5139025493</v>
       </c>
       <c r="G42" s="38" t="n">
         <f aca="false">G35-SUM(G38:G41)</f>
-        <v>10978.4050392288</v>
+        <v>16144.6370032288</v>
       </c>
       <c r="H42" s="2"/>
     </row>
@@ -6120,23 +6117,23 @@
       <c r="B43" s="2"/>
       <c r="C43" s="34" t="n">
         <f aca="false">IF(C25=0,0,C42/C25)</f>
-        <v>-4.04830236618059</v>
+        <v>-0.315792866778938</v>
       </c>
       <c r="D43" s="34" t="n">
         <f aca="false">IF(D25=0,0,D42/D25)</f>
-        <v>-0.271328469988929</v>
+        <v>0.665990029984332</v>
       </c>
       <c r="E43" s="34" t="n">
         <f aca="false">IF(E25=0,0,E42/E25)</f>
-        <v>0.396079563169408</v>
+        <v>0.842256485834526</v>
       </c>
       <c r="F43" s="34" t="n">
         <f aca="false">IF(F25=0,0,F42/F25)</f>
-        <v>0.542570745612598</v>
+        <v>0.88176887732771</v>
       </c>
       <c r="G43" s="34" t="n">
         <f aca="false">IF(G25=0,0,G42/G25)</f>
-        <v>0.612127686524311</v>
+        <v>0.900183520579547</v>
       </c>
       <c r="H43" s="2"/>
     </row>
@@ -6174,23 +6171,23 @@
       <c r="B45" s="2"/>
       <c r="C45" s="28" t="n">
         <f aca="false">C42-C44</f>
-        <v>-4101.48672832</v>
+        <v>-1739.81196165333</v>
       </c>
       <c r="D45" s="28" t="n">
         <f aca="false">C45+D42-D44</f>
-        <v>-5482.054614368</v>
+        <v>1648.864677632</v>
       </c>
       <c r="E45" s="28" t="n">
         <f aca="false">D45+E42-E44</f>
-        <v>-1116.812016928</v>
+        <v>10931.4791617387</v>
       </c>
       <c r="F45" s="28" t="n">
         <f aca="false">E45+F42-F44</f>
-        <v>7010.046222288</v>
+        <v>24138.993064288</v>
       </c>
       <c r="G45" s="28" t="n">
         <f aca="false">F45+G42-G44</f>
-        <v>17988.4512615168</v>
+        <v>40283.6300675168</v>
       </c>
       <c r="H45" s="17" t="s">
         <v>264</v>
@@ -6880,50 +6877,50 @@
       <c r="B9" s="2"/>
       <c r="C9" s="33" t="n">
         <f aca="false">IF(Rollout!C$7=0,0,MAX(1,ROUNDUP(Rollout!C$7/Assumptions!$C$76,0)))</f>
-        <v>75</v>
+        <v>3</v>
       </c>
       <c r="D9" s="33" t="n">
         <f aca="false">IF(Rollout!D$7=0,0,MAX(1,ROUNDUP(Rollout!D$7/Assumptions!$C$76,0)))</f>
-        <v>148</v>
+        <v>6</v>
       </c>
       <c r="E9" s="33" t="n">
         <f aca="false">IF(Rollout!E$7=0,0,MAX(1,ROUNDUP(Rollout!E$7/Assumptions!$C$76,0)))</f>
-        <v>205</v>
+        <v>9</v>
       </c>
       <c r="F9" s="33" t="n">
         <f aca="false">IF(Rollout!F$7=0,0,MAX(1,ROUNDUP(Rollout!F$7/Assumptions!$C$76,0)))</f>
-        <v>201</v>
+        <v>9</v>
       </c>
       <c r="G9" s="33" t="n">
         <f aca="false">IF(Rollout!G$7=0,0,MAX(1,ROUNDUP(Rollout!G$7/Assumptions!$C$76,0)))</f>
-        <v>199</v>
+        <v>8</v>
       </c>
       <c r="H9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>280</v>
+        <v>176</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="33" t="n">
         <f aca="false">IF(Rollout!C$7=0,0,MAX(1,ROUNDUP(Rollout!C$7/Assumptions!$C$77,0)))</f>
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="D10" s="33" t="n">
         <f aca="false">IF(Rollout!D$7=0,0,MAX(1,ROUNDUP(Rollout!D$7/Assumptions!$C$77,0)))</f>
-        <v>197</v>
+        <v>6</v>
       </c>
       <c r="E10" s="33" t="n">
         <f aca="false">IF(Rollout!E$7=0,0,MAX(1,ROUNDUP(Rollout!E$7/Assumptions!$C$77,0)))</f>
-        <v>274</v>
+        <v>9</v>
       </c>
       <c r="F10" s="33" t="n">
         <f aca="false">IF(Rollout!F$7=0,0,MAX(1,ROUNDUP(Rollout!F$7/Assumptions!$C$77,0)))</f>
-        <v>268</v>
+        <v>9</v>
       </c>
       <c r="G10" s="33" t="n">
         <f aca="false">IF(Rollout!G$7=0,0,MAX(1,ROUNDUP(Rollout!G$7/Assumptions!$C$77,0)))</f>
-        <v>265</v>
+        <v>8</v>
       </c>
       <c r="H10" s="2"/>
     </row>
@@ -6956,7 +6953,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="33" t="n">
@@ -6983,47 +6980,47 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="39" t="n">
         <f aca="false">SUM(C6:C12)</f>
-        <v>214</v>
+        <v>45</v>
       </c>
       <c r="D13" s="39" t="n">
         <f aca="false">SUM(D6:D12)</f>
-        <v>411</v>
+        <v>78</v>
       </c>
       <c r="E13" s="39" t="n">
         <f aca="false">SUM(E6:E12)</f>
-        <v>568</v>
+        <v>107</v>
       </c>
       <c r="F13" s="39" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>554</v>
+        <v>103</v>
       </c>
       <c r="G13" s="39" t="n">
         <f aca="false">SUM(G6:G12)</f>
-        <v>554</v>
+        <v>106</v>
       </c>
       <c r="H13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="33" t="n">
         <f aca="false">C13</f>
-        <v>214</v>
+        <v>45</v>
       </c>
       <c r="D14" s="33" t="n">
         <f aca="false">MAX(0,D13-C13)</f>
-        <v>197</v>
+        <v>33</v>
       </c>
       <c r="E14" s="33" t="n">
         <f aca="false">MAX(0,E13-D13)</f>
-        <v>157</v>
+        <v>29</v>
       </c>
       <c r="F14" s="33" t="n">
         <f aca="false">MAX(0,F13-E13)</f>
@@ -7031,7 +7028,7 @@
       </c>
       <c r="G14" s="33" t="n">
         <f aca="false">MAX(0,G13-F13)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H14" s="2"/>
     </row>
@@ -7047,7 +7044,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -7145,50 +7142,50 @@
       <c r="B20" s="2"/>
       <c r="C20" s="37" t="n">
         <f aca="false">C9*0.75*Assumptions!$C$83*(1+Assumptions!$C$73)*(1+Assumptions!$C$74)^0</f>
-        <v>4921875</v>
+        <v>196875</v>
       </c>
       <c r="D20" s="37" t="n">
         <f aca="false">(C9+D9)/2*Assumptions!$C$83*(1+Assumptions!$C$73)*(1+Assumptions!$C$74)^1</f>
-        <v>10048937.5</v>
+        <v>405562.5</v>
       </c>
       <c r="E20" s="37" t="n">
         <f aca="false">(D9+E9)/2*Assumptions!$C$83*(1+Assumptions!$C$73)*(1+Assumptions!$C$74)^2</f>
-        <v>16384274.375</v>
+        <v>696215.625</v>
       </c>
       <c r="F20" s="37" t="n">
         <f aca="false">(E9+F9)/2*Assumptions!$C$83*(1+Assumptions!$C$73)*(1+Assumptions!$C$74)^3</f>
-        <v>19409563.3375</v>
+        <v>860522.5125</v>
       </c>
       <c r="G20" s="37" t="n">
         <f aca="false">(F9+G9)/2*Assumptions!$C$83*(1+Assumptions!$C$73)*(1+Assumptions!$C$74)^4</f>
-        <v>19696404.175</v>
+        <v>837097.1774375</v>
       </c>
       <c r="H20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>280</v>
+        <v>176</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="37" t="n">
         <f aca="false">C10*0.75*Assumptions!$C$84*(1+Assumptions!$C$73)*(1+Assumptions!$C$74)^0</f>
-        <v>6093750</v>
+        <v>182812.5</v>
       </c>
       <c r="D21" s="37" t="n">
         <f aca="false">(C10+D10)/2*Assumptions!$C$84*(1+Assumptions!$C$73)*(1+Assumptions!$C$74)^1</f>
-        <v>12427593.75</v>
+        <v>376593.75</v>
       </c>
       <c r="E21" s="37" t="n">
         <f aca="false">(D10+E10)/2*Assumptions!$C$84*(1+Assumptions!$C$73)*(1+Assumptions!$C$74)^2</f>
-        <v>20299658.4375</v>
+        <v>646485.9375</v>
       </c>
       <c r="F21" s="37" t="n">
         <f aca="false">(E10+F10)/2*Assumptions!$C$84*(1+Assumptions!$C$73)*(1+Assumptions!$C$74)^3</f>
-        <v>24060482.63125</v>
+        <v>799056.61875</v>
       </c>
       <c r="G21" s="37" t="n">
         <f aca="false">(F10+G10)/2*Assumptions!$C$84*(1+Assumptions!$C$73)*(1+Assumptions!$C$74)^4</f>
-        <v>24370782.9515313</v>
+        <v>777304.52190625</v>
       </c>
       <c r="H21" s="2"/>
     </row>
@@ -7221,7 +7218,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="37" t="n">
@@ -7248,28 +7245,28 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="38" t="n">
         <f aca="false">SUM(C17:C23)</f>
-        <v>13710937.5</v>
+        <v>3075000</v>
       </c>
       <c r="D24" s="38" t="n">
         <f aca="false">SUM(D17:D23)</f>
-        <v>27282125</v>
+        <v>5587750</v>
       </c>
       <c r="E24" s="38" t="n">
         <f aca="false">SUM(E17:E23)</f>
-        <v>43934521.25</v>
+        <v>8593290</v>
       </c>
       <c r="F24" s="38" t="n">
         <f aca="false">SUM(F17:F23)</f>
-        <v>52259668.775</v>
+        <v>10449201.9375</v>
       </c>
       <c r="G24" s="38" t="n">
         <f aca="false">SUM(G17:G23)</f>
-        <v>53795803.9029688</v>
+        <v>11343018.4757813</v>
       </c>
       <c r="H24" s="2"/>
     </row>
@@ -7285,7 +7282,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -7322,7 +7319,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7334,7 +7331,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7378,7 +7375,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -7395,23 +7392,23 @@
       <c r="B6" s="2"/>
       <c r="C6" s="37" t="n">
         <f aca="false">Rollout!$C$5*'Unit Economics'!$C$29</f>
-        <v>512898</v>
+        <v>572685</v>
       </c>
       <c r="D6" s="37" t="n">
         <f aca="false">Rollout!$C$5*'Unit Economics'!$D$29+Rollout!$D$5*'Unit Economics'!$C$29</f>
-        <v>1507920.12</v>
+        <v>1683693.9</v>
       </c>
       <c r="E6" s="37" t="n">
         <f aca="false">Rollout!$C$5*'Unit Economics'!$E$29+Rollout!$D$5*'Unit Economics'!$D$29+Rollout!$E$5*'Unit Economics'!$C$29</f>
-        <v>2385488.598</v>
+        <v>2663557.935</v>
       </c>
       <c r="F6" s="37" t="n">
         <f aca="false">Rollout!$C$5*'Unit Economics'!$F$29+Rollout!$D$5*'Unit Economics'!$E$29+Rollout!$E$5*'Unit Economics'!$D$29+Rollout!$F$5*'Unit Economics'!$C$29</f>
-        <v>2745717.37932</v>
+        <v>3065777.5179</v>
       </c>
       <c r="G6" s="37" t="n">
         <f aca="false">Rollout!$C$5*'Unit Economics'!$G$29+Rollout!$D$5*'Unit Economics'!$F$29+Rollout!$E$5*'Unit Economics'!$E$29+Rollout!$F$5*'Unit Economics'!$D$29+Rollout!$G$5*'Unit Economics'!$C$29</f>
-        <v>2708563.0482</v>
+        <v>3024292.2165</v>
       </c>
       <c r="H6" s="2"/>
     </row>
@@ -7498,7 +7495,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="37" t="n">
@@ -7525,28 +7522,28 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="38" t="n">
         <f aca="false">SUM(C6:C10)</f>
-        <v>1079030.12496</v>
+        <v>1138817.12496</v>
       </c>
       <c r="D11" s="38" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>3441086.083104</v>
+        <v>3616859.863104</v>
       </c>
       <c r="E11" s="38" t="n">
         <f aca="false">SUM(E6:E10)</f>
-        <v>5871878.75716656</v>
+        <v>6149948.09416656</v>
       </c>
       <c r="F11" s="38" t="n">
         <f aca="false">SUM(F6:F10)</f>
-        <v>7397026.37408678</v>
+        <v>7717086.51266678</v>
       </c>
       <c r="G11" s="38" t="n">
         <f aca="false">SUM(G6:G10)</f>
-        <v>8007507.78225408</v>
+        <v>8323236.95055408</v>
       </c>
       <c r="H11" s="2"/>
     </row>
@@ -7562,7 +7559,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -7574,88 +7571,88 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="9" t="n">
         <f aca="false">Headcount!C20</f>
-        <v>4921875</v>
+        <v>196875</v>
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">Headcount!D20</f>
-        <v>10048937.5</v>
+        <v>405562.5</v>
       </c>
       <c r="E14" s="9" t="n">
         <f aca="false">Headcount!E20</f>
-        <v>16384274.375</v>
+        <v>696215.625</v>
       </c>
       <c r="F14" s="9" t="n">
         <f aca="false">Headcount!F20</f>
-        <v>19409563.3375</v>
+        <v>860522.5125</v>
       </c>
       <c r="G14" s="9" t="n">
         <f aca="false">Headcount!G20</f>
-        <v>19696404.175</v>
+        <v>837097.1774375</v>
       </c>
       <c r="H14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="9" t="n">
         <f aca="false">Headcount!C21</f>
-        <v>6093750</v>
+        <v>182812.5</v>
       </c>
       <c r="D15" s="9" t="n">
         <f aca="false">Headcount!D21</f>
-        <v>12427593.75</v>
+        <v>376593.75</v>
       </c>
       <c r="E15" s="9" t="n">
         <f aca="false">Headcount!E21</f>
-        <v>20299658.4375</v>
+        <v>646485.9375</v>
       </c>
       <c r="F15" s="9" t="n">
         <f aca="false">Headcount!F21</f>
-        <v>24060482.63125</v>
+        <v>799056.61875</v>
       </c>
       <c r="G15" s="9" t="n">
         <f aca="false">Headcount!G21</f>
-        <v>24370782.9515313</v>
+        <v>777304.52190625</v>
       </c>
       <c r="H15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="37" t="n">
         <f aca="false">(Rollout!$C$5*'Unit Economics'!$C$27)*Assumptions!$C$75</f>
-        <v>54186.3</v>
+        <v>0</v>
       </c>
       <c r="D16" s="37" t="n">
         <f aca="false">(Rollout!$C$5*'Unit Economics'!$D$27+Rollout!$D$5*'Unit Economics'!$C$27)*Assumptions!$C$75</f>
-        <v>722094.156</v>
+        <v>0</v>
       </c>
       <c r="E16" s="37" t="n">
         <f aca="false">(Rollout!$C$5*'Unit Economics'!$E$27+Rollout!$D$5*'Unit Economics'!$D$27+Rollout!$E$5*'Unit Economics'!$C$27)*Assumptions!$C$75</f>
-        <v>2105376.4053</v>
+        <v>0</v>
       </c>
       <c r="F16" s="37" t="n">
         <f aca="false">(Rollout!$C$5*'Unit Economics'!$F$27+Rollout!$D$5*'Unit Economics'!$E$27+Rollout!$E$5*'Unit Economics'!$D$27+Rollout!$F$5*'Unit Economics'!$C$27)*Assumptions!$C$75</f>
-        <v>3959188.281216</v>
+        <v>0</v>
       </c>
       <c r="G16" s="37" t="n">
         <f aca="false">(Rollout!$C$5*'Unit Economics'!$G$27+Rollout!$D$5*'Unit Economics'!$F$27+Rollout!$E$5*'Unit Economics'!$E$27+Rollout!$F$5*'Unit Economics'!$D$27+Rollout!$G$5*'Unit Economics'!$C$27)*Assumptions!$C$75</f>
-        <v>5575476.28806</v>
+        <v>0</v>
       </c>
       <c r="H16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="9" t="n">
@@ -7682,7 +7679,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="9" t="n">
@@ -7709,7 +7706,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="37" t="n">
@@ -7790,7 +7787,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="9" t="n">
@@ -7817,7 +7814,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="9" t="n">
@@ -7844,7 +7841,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="9" t="n">
@@ -7871,7 +7868,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="37" t="n">
@@ -7898,55 +7895,55 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="37" t="n">
         <f aca="false">Headcount!C13*Assumptions!$C$99</f>
-        <v>642000</v>
+        <v>135000</v>
       </c>
       <c r="D26" s="37" t="n">
         <f aca="false">Headcount!D13*Assumptions!$C$99</f>
-        <v>1233000</v>
+        <v>234000</v>
       </c>
       <c r="E26" s="37" t="n">
         <f aca="false">Headcount!E13*Assumptions!$C$99</f>
-        <v>1704000</v>
+        <v>321000</v>
       </c>
       <c r="F26" s="37" t="n">
         <f aca="false">Headcount!F13*Assumptions!$C$99</f>
-        <v>1662000</v>
+        <v>309000</v>
       </c>
       <c r="G26" s="37" t="n">
         <f aca="false">Headcount!G13*Assumptions!$C$99</f>
-        <v>1662000</v>
+        <v>318000</v>
       </c>
       <c r="H26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="38" t="n">
         <f aca="false">SUM(C14:C26)</f>
-        <v>19533435.8</v>
+        <v>8336312</v>
       </c>
       <c r="D27" s="38" t="n">
         <f aca="false">SUM(D14:D26)</f>
-        <v>35251246.196</v>
+        <v>11835777.04</v>
       </c>
       <c r="E27" s="38" t="n">
         <f aca="false">SUM(E14:E26)</f>
-        <v>53651300.2873</v>
+        <v>14821692.632</v>
       </c>
       <c r="F27" s="38" t="n">
         <f aca="false">SUM(F14:F26)</f>
-        <v>60382503.313656</v>
+        <v>13259848.19494</v>
       </c>
       <c r="G27" s="38" t="n">
         <f aca="false">SUM(G14:G26)</f>
-        <v>63505731.7231888</v>
+        <v>14133470.0079413</v>
       </c>
       <c r="H27" s="2"/>
     </row>
@@ -7977,7 +7974,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7989,7 +7986,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8033,7 +8030,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="28" t="n">
@@ -8060,55 +8057,55 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="9" t="n">
         <f aca="false">Costs!C11</f>
-        <v>1079030.12496</v>
+        <v>1138817.12496</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">Costs!D11</f>
-        <v>3441086.083104</v>
+        <v>3616859.863104</v>
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">Costs!E11</f>
-        <v>5871878.75716656</v>
+        <v>6149948.09416656</v>
       </c>
       <c r="F6" s="9" t="n">
         <f aca="false">Costs!F11</f>
-        <v>7397026.37408678</v>
+        <v>7717086.51266678</v>
       </c>
       <c r="G6" s="9" t="n">
         <f aca="false">Costs!G11</f>
-        <v>8007507.78225408</v>
+        <v>8323236.95055408</v>
       </c>
       <c r="H6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="38" t="n">
         <f aca="false">C5-C6</f>
-        <v>819163.11504</v>
+        <v>759376.11504</v>
       </c>
       <c r="D7" s="38" t="n">
         <f aca="false">D5-D6</f>
-        <v>13721644.852896</v>
+        <v>13545871.072896</v>
       </c>
       <c r="E7" s="38" t="n">
         <f aca="false">E5-E6</f>
-        <v>43995470.3364734</v>
+        <v>43717400.9994734</v>
       </c>
       <c r="F7" s="38" t="n">
         <f aca="false">F5-F6</f>
-        <v>82981182.0693692</v>
+        <v>82661121.9307892</v>
       </c>
       <c r="G7" s="38" t="n">
         <f aca="false">G5-G6</f>
-        <v>117546667.707626</v>
+        <v>117230938.539326</v>
       </c>
       <c r="H7" s="2"/>
     </row>
@@ -8119,23 +8116,23 @@
       <c r="B8" s="2"/>
       <c r="C8" s="34" t="n">
         <f aca="false">IF(C5=0,0,C7/C5)</f>
-        <v>0.431548852760639</v>
+        <v>0.400052059525826</v>
       </c>
       <c r="D8" s="34" t="n">
         <f aca="false">IF(D5=0,0,D7/D5)</f>
-        <v>0.799502416256723</v>
+        <v>0.789260818887664</v>
       </c>
       <c r="E8" s="34" t="n">
         <f aca="false">IF(E5=0,0,E7/E5)</f>
-        <v>0.88225003205724</v>
+        <v>0.876673851609431</v>
       </c>
       <c r="F8" s="34" t="n">
         <f aca="false">IF(F5=0,0,F7/F5)</f>
-        <v>0.918154757640337</v>
+        <v>0.914613415716302</v>
       </c>
       <c r="G8" s="34" t="n">
         <f aca="false">IF(G5=0,0,G7/G5)</f>
-        <v>0.936222688325491</v>
+        <v>0.933708003592243</v>
       </c>
       <c r="H8" s="2"/>
     </row>
@@ -8151,55 +8148,55 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="9" t="n">
         <f aca="false">Costs!C14</f>
-        <v>4921875</v>
+        <v>196875</v>
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">Costs!D14</f>
-        <v>10048937.5</v>
+        <v>405562.5</v>
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">Costs!E14</f>
-        <v>16384274.375</v>
+        <v>696215.625</v>
       </c>
       <c r="F10" s="9" t="n">
         <f aca="false">Costs!F14</f>
-        <v>19409563.3375</v>
+        <v>860522.5125</v>
       </c>
       <c r="G10" s="9" t="n">
         <f aca="false">Costs!G14</f>
-        <v>19696404.175</v>
+        <v>837097.1774375</v>
       </c>
       <c r="H10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="9" t="n">
         <f aca="false">Costs!C15+Costs!C16+Costs!C17+Costs!C18+Costs!C19+Costs!C20+Costs!C21</f>
-        <v>12878310.8</v>
+        <v>6913187</v>
       </c>
       <c r="D11" s="9" t="n">
         <f aca="false">Costs!D15+Costs!D16+Costs!D17+Costs!D18+Costs!D19+Costs!D20+Costs!D21</f>
-        <v>22004683.696</v>
+        <v>9231589.54</v>
       </c>
       <c r="E11" s="9" t="n">
         <f aca="false">Costs!E15+Costs!E16+Costs!E17+Costs!E18+Costs!E19+Costs!E20+Costs!E21</f>
-        <v>32503247.1623</v>
+        <v>10744698.257</v>
       </c>
       <c r="F11" s="9" t="n">
         <f aca="false">Costs!F15+Costs!F16+Costs!F17+Costs!F18+Costs!F19+Costs!F20+Costs!F21</f>
-        <v>34953313.038656</v>
+        <v>7732698.74494</v>
       </c>
       <c r="G11" s="9" t="n">
         <f aca="false">Costs!G15+Costs!G16+Costs!G17+Costs!G18+Costs!G19+Costs!G20+Costs!G21</f>
-        <v>36545517.7278138</v>
+        <v>7376563.01012875</v>
       </c>
       <c r="H11" s="2"/>
     </row>
@@ -8232,55 +8229,55 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="9" t="n">
         <f aca="false">Costs!C23+Costs!C24+Costs!C25+Costs!C26</f>
-        <v>1255125</v>
+        <v>748125</v>
       </c>
       <c r="D13" s="9" t="n">
         <f aca="false">Costs!D23+Costs!D24+Costs!D25+Costs!D26</f>
-        <v>2322125</v>
+        <v>1323125</v>
       </c>
       <c r="E13" s="9" t="n">
         <f aca="false">Costs!E23+Costs!E24+Costs!E25+Costs!E26</f>
-        <v>3298410.625</v>
+        <v>1915410.625</v>
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">Costs!F23+Costs!F24+Costs!F25+Costs!F26</f>
-        <v>3813684.30625</v>
+        <v>2460684.30625</v>
       </c>
       <c r="G13" s="9" t="n">
         <f aca="false">Costs!G23+Costs!G24+Costs!G25+Costs!G26</f>
-        <v>4274177.0438125</v>
+        <v>2930177.0438125</v>
       </c>
       <c r="H13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="40" t="n">
         <f aca="false">SUM(C10:C13)</f>
-        <v>19533435.8</v>
+        <v>8336312</v>
       </c>
       <c r="D14" s="40" t="n">
         <f aca="false">SUM(D10:D13)</f>
-        <v>35251246.196</v>
+        <v>11835777.04</v>
       </c>
       <c r="E14" s="40" t="n">
         <f aca="false">SUM(E10:E13)</f>
-        <v>53651300.2873</v>
+        <v>14821692.632</v>
       </c>
       <c r="F14" s="40" t="n">
         <f aca="false">SUM(F10:F13)</f>
-        <v>60382503.313656</v>
+        <v>13259848.19494</v>
       </c>
       <c r="G14" s="40" t="n">
         <f aca="false">SUM(G10:G13)</f>
-        <v>63505731.7231888</v>
+        <v>14133470.0079413</v>
       </c>
       <c r="H14" s="2"/>
     </row>
@@ -8296,28 +8293,28 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="28" t="n">
         <f aca="false">C7-C14</f>
-        <v>-18714272.68496</v>
+        <v>-7576935.88496</v>
       </c>
       <c r="D16" s="28" t="n">
         <f aca="false">D7-D14</f>
-        <v>-21529601.343104</v>
+        <v>1710094.032896</v>
       </c>
       <c r="E16" s="28" t="n">
         <f aca="false">E7-E14</f>
-        <v>-9655829.95082656</v>
+        <v>28895708.3674734</v>
       </c>
       <c r="F16" s="28" t="n">
         <f aca="false">F7-F14</f>
-        <v>22598678.7557132</v>
+        <v>69401273.7358492</v>
       </c>
       <c r="G16" s="28" t="n">
         <f aca="false">G7-G14</f>
-        <v>54040935.9844372</v>
+        <v>103097468.531385</v>
       </c>
       <c r="H16" s="2"/>
     </row>
@@ -8328,42 +8325,42 @@
       <c r="B17" s="2"/>
       <c r="C17" s="34" t="n">
         <f aca="false">IF(C5=0,0,C16/C5)</f>
-        <v>-9.85899237790985</v>
+        <v>-3.99165676354426</v>
       </c>
       <c r="D17" s="34" t="n">
         <f aca="false">IF(D5=0,0,D16/D5)</f>
-        <v>-1.25443913462188</v>
+        <v>0.0996399721741811</v>
       </c>
       <c r="E17" s="34" t="n">
         <f aca="false">IF(E5=0,0,E16/E5)</f>
-        <v>-0.193630303722282</v>
+        <v>0.579451462583535</v>
       </c>
       <c r="F17" s="34" t="n">
         <f aca="false">IF(F5=0,0,F16/F5)</f>
-        <v>0.250045659732808</v>
+        <v>0.76789831233786</v>
       </c>
       <c r="G17" s="34" t="n">
         <f aca="false">IF(G5=0,0,G16/G5)</f>
-        <v>0.430419265417366</v>
+        <v>0.82113930603363</v>
       </c>
       <c r="H17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="37" t="n">
         <f aca="false">Headcount!C14*Assumptions!$C$100</f>
-        <v>535000</v>
+        <v>112500</v>
       </c>
       <c r="D18" s="37" t="n">
         <f aca="false">Headcount!D14*Assumptions!$C$100</f>
-        <v>492500</v>
+        <v>82500</v>
       </c>
       <c r="E18" s="37" t="n">
         <f aca="false">Headcount!E14*Assumptions!$C$100</f>
-        <v>392500</v>
+        <v>72500</v>
       </c>
       <c r="F18" s="37" t="n">
         <f aca="false">Headcount!F14*Assumptions!$C$100</f>
@@ -8371,67 +8368,67 @@
       </c>
       <c r="G18" s="37" t="n">
         <f aca="false">Headcount!G14*Assumptions!$C$100</f>
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="H18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="37" t="n">
         <f aca="false">(C18)/Assumptions!$C$101</f>
-        <v>178333.333333333</v>
+        <v>37500</v>
       </c>
       <c r="D19" s="37" t="n">
         <f aca="false">(C18+D18)/Assumptions!$C$101</f>
-        <v>342500</v>
+        <v>65000</v>
       </c>
       <c r="E19" s="37" t="n">
         <f aca="false">(C18+D18+E18)/Assumptions!$C$101</f>
-        <v>473333.333333333</v>
+        <v>89166.6666666667</v>
       </c>
       <c r="F19" s="37" t="n">
         <f aca="false">(D18+E18+F18)/Assumptions!$C$101</f>
-        <v>295000</v>
+        <v>51666.6666666667</v>
       </c>
       <c r="G19" s="37" t="n">
         <f aca="false">(E18+F18+G18)/Assumptions!$C$101</f>
-        <v>130833.333333333</v>
+        <v>26666.6666666667</v>
       </c>
       <c r="H19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="28" t="n">
         <f aca="false">C16-C19</f>
-        <v>-18892606.0182933</v>
+        <v>-7614435.88496</v>
       </c>
       <c r="D20" s="28" t="n">
         <f aca="false">D16-D19</f>
-        <v>-21872101.343104</v>
+        <v>1645094.032896</v>
       </c>
       <c r="E20" s="28" t="n">
         <f aca="false">E16-E19</f>
-        <v>-10129163.2841599</v>
+        <v>28806541.7008068</v>
       </c>
       <c r="F20" s="28" t="n">
         <f aca="false">F16-F19</f>
-        <v>22303678.7557132</v>
+        <v>69349607.0691826</v>
       </c>
       <c r="G20" s="28" t="n">
         <f aca="false">G16-G19</f>
-        <v>53910102.6511038</v>
+        <v>103070801.864718</v>
       </c>
       <c r="H20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="37" t="n">
@@ -8440,25 +8437,25 @@
       </c>
       <c r="D21" s="37" t="n">
         <f aca="false">C23</f>
-        <v>18892606.0182933</v>
+        <v>7614435.88496</v>
       </c>
       <c r="E21" s="37" t="n">
         <f aca="false">D23</f>
-        <v>40764707.3613973</v>
+        <v>5969341.852064</v>
       </c>
       <c r="F21" s="37" t="n">
         <f aca="false">E23</f>
-        <v>50893870.6455572</v>
+        <v>0</v>
       </c>
       <c r="G21" s="37" t="n">
         <f aca="false">F23</f>
-        <v>28590191.889844</v>
+        <v>0</v>
       </c>
       <c r="H21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="37" t="n">
@@ -8471,38 +8468,38 @@
       </c>
       <c r="E22" s="37" t="n">
         <f aca="false">MAX(0,E20-E21)</f>
-        <v>0</v>
+        <v>22837199.8487428</v>
       </c>
       <c r="F22" s="37" t="n">
         <f aca="false">MAX(0,F20-F21)</f>
-        <v>0</v>
+        <v>69349607.0691826</v>
       </c>
       <c r="G22" s="37" t="n">
         <f aca="false">MAX(0,G20-G21)</f>
-        <v>25319910.7612598</v>
+        <v>103070801.864718</v>
       </c>
       <c r="H22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="37" t="n">
         <f aca="false">MAX(0,C21-MAX(0,C20))+MAX(0,-C20)</f>
-        <v>18892606.0182933</v>
+        <v>7614435.88496</v>
       </c>
       <c r="D23" s="37" t="n">
         <f aca="false">MAX(0,D21-MAX(0,D20))+MAX(0,-D20)</f>
-        <v>40764707.3613973</v>
+        <v>5969341.852064</v>
       </c>
       <c r="E23" s="37" t="n">
         <f aca="false">MAX(0,E21-MAX(0,E20))+MAX(0,-E20)</f>
-        <v>50893870.6455572</v>
+        <v>0</v>
       </c>
       <c r="F23" s="37" t="n">
         <f aca="false">MAX(0,F21-MAX(0,F20))+MAX(0,-F20)</f>
-        <v>28590191.889844</v>
+        <v>0</v>
       </c>
       <c r="G23" s="37" t="n">
         <f aca="false">MAX(0,G21-MAX(0,G20))+MAX(0,-G20)</f>
@@ -8512,7 +8509,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="37" t="n">
@@ -8525,42 +8522,42 @@
       </c>
       <c r="E24" s="37" t="n">
         <f aca="false">E22*Assumptions!$C$104</f>
-        <v>0</v>
+        <v>5709299.96218569</v>
       </c>
       <c r="F24" s="37" t="n">
         <f aca="false">F22*Assumptions!$C$104</f>
-        <v>0</v>
+        <v>17337401.7672956</v>
       </c>
       <c r="G24" s="37" t="n">
         <f aca="false">G22*Assumptions!$C$104</f>
-        <v>6329977.69031496</v>
+        <v>25767700.4661795</v>
       </c>
       <c r="H24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="38" t="n">
         <f aca="false">C20-C24</f>
-        <v>-18892606.0182933</v>
+        <v>-7614435.88496</v>
       </c>
       <c r="D25" s="38" t="n">
         <f aca="false">D20-D24</f>
-        <v>-21872101.343104</v>
+        <v>1645094.032896</v>
       </c>
       <c r="E25" s="38" t="n">
         <f aca="false">E20-E24</f>
-        <v>-10129163.2841599</v>
+        <v>23097241.7386211</v>
       </c>
       <c r="F25" s="38" t="n">
         <f aca="false">F20-F24</f>
-        <v>22303678.7557132</v>
+        <v>52012205.3018869</v>
       </c>
       <c r="G25" s="38" t="n">
         <f aca="false">G20-G24</f>
-        <v>47580124.9607889</v>
+        <v>77303101.3985385</v>
       </c>
       <c r="H25" s="2"/>
     </row>
@@ -8591,7 +8588,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -8603,7 +8600,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8647,34 +8644,34 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="9" t="n">
         <f aca="false">'P&amp;L'!C16</f>
-        <v>-18714272.68496</v>
+        <v>-7576935.88496</v>
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">'P&amp;L'!D16</f>
-        <v>-21529601.343104</v>
+        <v>1710094.032896</v>
       </c>
       <c r="E5" s="9" t="n">
         <f aca="false">'P&amp;L'!E16</f>
-        <v>-9655829.95082656</v>
+        <v>28895708.3674734</v>
       </c>
       <c r="F5" s="9" t="n">
         <f aca="false">'P&amp;L'!F16</f>
-        <v>22598678.7557132</v>
+        <v>69401273.7358492</v>
       </c>
       <c r="G5" s="9" t="n">
         <f aca="false">'P&amp;L'!G16</f>
-        <v>54040935.9844372</v>
+        <v>103097468.531385</v>
       </c>
       <c r="H5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="9" t="n">
@@ -8687,34 +8684,34 @@
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">-'P&amp;L'!E24</f>
-        <v>-0</v>
+        <v>-5709299.96218569</v>
       </c>
       <c r="F6" s="9" t="n">
         <f aca="false">-'P&amp;L'!F24</f>
-        <v>-0</v>
+        <v>-17337401.7672956</v>
       </c>
       <c r="G6" s="9" t="n">
         <f aca="false">-'P&amp;L'!G24</f>
-        <v>-6329977.69031496</v>
+        <v>-25767700.4661795</v>
       </c>
       <c r="H6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="9" t="n">
         <f aca="false">-'P&amp;L'!C18</f>
-        <v>-535000</v>
+        <v>-112500</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">-'P&amp;L'!D18</f>
-        <v>-492500</v>
+        <v>-82500</v>
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">-'P&amp;L'!E18</f>
-        <v>-392500</v>
+        <v>-72500</v>
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">-'P&amp;L'!F18</f>
@@ -8722,13 +8719,13 @@
       </c>
       <c r="G7" s="9" t="n">
         <f aca="false">-'P&amp;L'!G18</f>
-        <v>-0</v>
+        <v>-7500</v>
       </c>
       <c r="H7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="37" t="n">
@@ -8755,28 +8752,28 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="38" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>-19306218.48216</v>
+        <v>-7746381.68216</v>
       </c>
       <c r="D9" s="38" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>-22480037.473984</v>
+        <v>1169657.902016</v>
       </c>
       <c r="E9" s="38" t="n">
         <f aca="false">SUM(E5:E8)</f>
-        <v>-11029468.4955558</v>
+        <v>22132769.8605585</v>
       </c>
       <c r="F9" s="38" t="n">
         <f aca="false">SUM(F5:F8)</f>
-        <v>21383352.9752188</v>
+        <v>50848546.1880591</v>
       </c>
       <c r="G9" s="38" t="n">
         <f aca="false">SUM(G5:G8)</f>
-        <v>46655679.2827295</v>
+        <v>76266989.0538125</v>
       </c>
       <c r="H9" s="2"/>
     </row>
@@ -8787,11 +8784,11 @@
       <c r="B10" s="2"/>
       <c r="C10" s="9" t="n">
         <f aca="false">Assumptions!C$109</f>
-        <v>25000000</v>
+        <v>10000000</v>
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">Assumptions!D$109</f>
-        <v>35000000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">Assumptions!E$109</f>
@@ -8809,34 +8806,34 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="37" t="n">
         <f aca="false">C9+C10</f>
-        <v>5693781.51784</v>
+        <v>2253618.31784</v>
       </c>
       <c r="D11" s="37" t="n">
         <f aca="false">D9+D10</f>
-        <v>12519962.526016</v>
+        <v>1169657.902016</v>
       </c>
       <c r="E11" s="37" t="n">
         <f aca="false">E9+E10</f>
-        <v>-11029468.4955558</v>
+        <v>22132769.8605585</v>
       </c>
       <c r="F11" s="37" t="n">
         <f aca="false">F9+F10</f>
-        <v>21383352.9752188</v>
+        <v>50848546.1880591</v>
       </c>
       <c r="G11" s="37" t="n">
         <f aca="false">G9+G10</f>
-        <v>46655679.2827295</v>
+        <v>76266989.0538125</v>
       </c>
       <c r="H11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="37" t="n">
@@ -8845,52 +8842,52 @@
       </c>
       <c r="D12" s="37" t="n">
         <f aca="false">C13</f>
-        <v>5943781.51784</v>
+        <v>2503618.31784</v>
       </c>
       <c r="E12" s="37" t="n">
         <f aca="false">D13</f>
-        <v>18463744.043856</v>
+        <v>3673276.219856</v>
       </c>
       <c r="F12" s="37" t="n">
         <f aca="false">E13</f>
-        <v>7434275.54830025</v>
+        <v>25806046.0804145</v>
       </c>
       <c r="G12" s="37" t="n">
         <f aca="false">F13</f>
-        <v>28817628.523519</v>
+        <v>76654592.2684737</v>
       </c>
       <c r="H12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="38" t="n">
         <f aca="false">C12+C11</f>
-        <v>5943781.51784</v>
+        <v>2503618.31784</v>
       </c>
       <c r="D13" s="38" t="n">
         <f aca="false">D12+D11</f>
-        <v>18463744.043856</v>
+        <v>3673276.219856</v>
       </c>
       <c r="E13" s="38" t="n">
         <f aca="false">E12+E11</f>
-        <v>7434275.54830025</v>
+        <v>25806046.0804145</v>
       </c>
       <c r="F13" s="38" t="n">
         <f aca="false">F12+F11</f>
-        <v>28817628.523519</v>
+        <v>76654592.2684737</v>
       </c>
       <c r="G13" s="38" t="n">
         <f aca="false">G12+G11</f>
-        <v>75473307.8062485</v>
+        <v>152921581.322286</v>
       </c>
       <c r="H13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="41" t="n">
@@ -8927,12 +8924,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="28" t="n">
         <f aca="false">MIN(C13:G13)</f>
-        <v>5943781.51784</v>
+        <v>2503618.31784</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
@@ -8942,19 +8939,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="28" t="n">
         <f aca="false">-MIN(0,C9,C9+D9,C9+D9+E9,C9+D9+E9+F9,C9+D9+E9+F9+G9)</f>
-        <v>52815724.4516998</v>
+        <v>7746381.68216</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="17" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>